<commit_message>
add LNG locations for mapping
</commit_message>
<xml_diff>
--- a/01_data/01_input_data/01_raw/01_Russian_War_Case/2411_GIE_LNG_Database_2025.xlsx
+++ b/01_data/01_input_data/01_raw/01_Russian_War_Case/2411_GIE_LNG_Database_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28429"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="28526"/>
   <workbookPr codeName="ThisWorkbook" defaultThemeVersion="124226"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Downloads\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\jfg.eco\Documents\GitHub\hydrogen_grid\01_data\01_input_data\01_raw\01_Russian_War_Case\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F16CFAB-5F55-42FC-94A6-46BD4D486418}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3B1DE247-27BA-43D4-B38E-F6CB36CD634B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-790" yWindow="0" windowWidth="8170" windowHeight="10170" firstSheet="1" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Import Terminals" sheetId="2" r:id="rId1"/>
@@ -1102,7 +1102,7 @@
     <t>including planneduntil 2035</t>
   </si>
   <si>
-    <t>Operational in 20242</t>
+    <t>Operational in 2024</t>
   </si>
 </sst>
 </file>
@@ -2237,7 +2237,7 @@
   </cellStyles>
   <dxfs count="5">
     <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
+      <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
       <numFmt numFmtId="2" formatCode="0.00"/>
@@ -2249,7 +2249,7 @@
       <numFmt numFmtId="2" formatCode="0.00"/>
     </dxf>
     <dxf>
-      <numFmt numFmtId="2" formatCode="0.00"/>
+      <numFmt numFmtId="0" formatCode="General"/>
     </dxf>
   </dxfs>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
@@ -6788,19 +6788,19 @@
   <autoFilter ref="B2:G26" xr:uid="{FF0AA701-883C-4FE2-873B-9C1A6221675F}"/>
   <tableColumns count="6">
     <tableColumn id="1" xr3:uid="{E567D681-9923-4237-B4F4-1466763A05FB}" name="Country"/>
-    <tableColumn id="6" xr3:uid="{30E9D74D-D363-4539-B18D-26B1FB6CD0CF}" name="Operational in 2021" dataDxfId="0">
+    <tableColumn id="6" xr3:uid="{30E9D74D-D363-4539-B18D-26B1FB6CD0CF}" name="Operational in 2021" dataDxfId="4">
       <calculatedColumnFormula>SUMIFS('Import Terminals'!$J$4:$J$77,'Import Terminals'!$A$4:$A$77,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$77,"operational",'Import Terminals'!$F$4:$F$77,"&lt;2022")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="2" xr3:uid="{6EBC0BA6-0EAD-4F87-A6B7-74F1999034D0}" name="Operational in 20242" dataDxfId="1">
+    <tableColumn id="2" xr3:uid="{6EBC0BA6-0EAD-4F87-A6B7-74F1999034D0}" name="Operational in 2024" dataDxfId="3">
       <calculatedColumnFormula>SUMIFS('Import Terminals'!$J$4:$J$77,'Import Terminals'!$A$4:$A$77,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$77,"operational",'Import Terminals'!$F$4:$F$77,"&lt;2025")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="3" xr3:uid="{F048872F-1DE8-4CAD-BF14-298B9BA60C55}" name="including under construction" dataDxfId="4">
+    <tableColumn id="3" xr3:uid="{F048872F-1DE8-4CAD-BF14-298B9BA60C55}" name="including under construction" dataDxfId="2">
       <calculatedColumnFormula>SUMIFS('Import Terminals'!$J$4:$J$77,'Import Terminals'!$A$4:$A$77,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$77,"operational",'Import Terminals'!$F$4:$F$77,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$77,'Import Terminals'!$A$4:$A$77,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$77,"under construction",'Import Terminals'!$F$4:$F$77,"&lt;2025")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="4" xr3:uid="{085B9AC4-9974-4CCB-8D60-234617C1C0D3}" name="including planneduntil 2025" dataDxfId="3">
+    <tableColumn id="4" xr3:uid="{085B9AC4-9974-4CCB-8D60-234617C1C0D3}" name="including planneduntil 2025" dataDxfId="1">
       <calculatedColumnFormula>SUMIFS('Import Terminals'!$J$4:$J$77,'Import Terminals'!$A$4:$A$77,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$77,"operational",'Import Terminals'!$F$4:$F$77,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$77,'Import Terminals'!$A$4:$A$77,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$77,"under construction",'Import Terminals'!$F$4:$F$77,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$77,'Import Terminals'!$A$4:$A$77,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$77,"planned",'Import Terminals'!$F$4:$F$77,"&lt;2025")</calculatedColumnFormula>
     </tableColumn>
-    <tableColumn id="5" xr3:uid="{490E5E38-720F-4821-9088-8C8EA4E48F3D}" name="including planneduntil 2035" dataDxfId="2">
+    <tableColumn id="5" xr3:uid="{490E5E38-720F-4821-9088-8C8EA4E48F3D}" name="including planneduntil 2035" dataDxfId="0">
       <calculatedColumnFormula>SUMIFS('Import Terminals'!$J$4:$J$77,'Import Terminals'!$A$4:$A$77,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$77,"operational",'Import Terminals'!$F$4:$F$77,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$77,'Import Terminals'!$A$4:$A$77,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$77,"under construction",'Import Terminals'!$F$4:$F$77,"&lt;2025")+SUMIFS('Import Terminals'!$J$4:$J$77,'Import Terminals'!$A$4:$A$77,Table1[[#This Row],[Country]],'Import Terminals'!$D$4:$D$77,"planned",'Import Terminals'!$F$4:$F$77,"&lt;2035")</calculatedColumnFormula>
     </tableColumn>
   </tableColumns>
@@ -7106,7 +7106,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <sheetPr codeName="Sheet1" filterMode="1">
+  <sheetPr codeName="Sheet1">
     <tabColor rgb="FF0070C0"/>
   </sheetPr>
   <dimension ref="A1:T77"/>
@@ -7231,7 +7231,7 @@
         <v>20</v>
       </c>
     </row>
-    <row r="4" spans="1:20" ht="14.5" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:20" ht="14.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A4" s="62" t="s">
         <v>21</v>
       </c>
@@ -7267,7 +7267,7 @@
       <c r="S4" s="63"/>
       <c r="T4" s="66"/>
     </row>
-    <row r="5" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A5" s="106" t="s">
         <v>28</v>
       </c>
@@ -7326,7 +7326,7 @@
         <v>36</v>
       </c>
     </row>
-    <row r="6" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="6" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A6" s="106" t="s">
         <v>28</v>
       </c>
@@ -7368,7 +7368,7 @@
       <c r="S6" s="112"/>
       <c r="T6" s="111"/>
     </row>
-    <row r="7" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="7" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A7" s="106" t="s">
         <v>28</v>
       </c>
@@ -7410,7 +7410,7 @@
       <c r="S7" s="112"/>
       <c r="T7" s="111"/>
     </row>
-    <row r="8" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="8" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A8" s="106" t="s">
         <v>39</v>
       </c>
@@ -7468,7 +7468,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="9" spans="1:20" s="4" customFormat="1" ht="13.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:20" s="4" customFormat="1" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A9" s="113" t="s">
         <v>39</v>
       </c>
@@ -7526,7 +7526,7 @@
         <v>42</v>
       </c>
     </row>
-    <row r="10" spans="1:20" s="4" customFormat="1" ht="13.9" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:20" s="4" customFormat="1" ht="13.9" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A10" s="113" t="s">
         <v>44</v>
       </c>
@@ -7572,7 +7572,7 @@
         <v>48</v>
       </c>
     </row>
-    <row r="11" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A11" s="113" t="s">
         <v>49</v>
       </c>
@@ -7608,7 +7608,7 @@
       <c r="S11" s="115"/>
       <c r="T11" s="119"/>
     </row>
-    <row r="12" spans="1:20" s="4" customFormat="1" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:20" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A12" s="113" t="s">
         <v>49</v>
       </c>
@@ -7652,7 +7652,7 @@
         <v>55</v>
       </c>
     </row>
-    <row r="13" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A13" s="113" t="s">
         <v>56</v>
       </c>
@@ -7698,7 +7698,7 @@
         <v>58</v>
       </c>
     </row>
-    <row r="14" spans="1:20" s="4" customFormat="1" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="14" spans="1:20" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A14" s="106" t="s">
         <v>56</v>
       </c>
@@ -7740,7 +7740,7 @@
         <v>60</v>
       </c>
     </row>
-    <row r="15" spans="1:20" s="4" customFormat="1" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="15" spans="1:20" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A15" s="106" t="s">
         <v>61</v>
       </c>
@@ -7796,7 +7796,7 @@
         <v>64</v>
       </c>
     </row>
-    <row r="16" spans="1:20" s="4" customFormat="1" ht="12.75" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="16" spans="1:20" s="4" customFormat="1" ht="12.75" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A16" s="106" t="s">
         <v>65</v>
       </c>
@@ -7854,7 +7854,7 @@
         <v>69</v>
       </c>
     </row>
-    <row r="17" spans="1:20" s="4" customFormat="1" ht="13.15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="17" spans="1:20" s="4" customFormat="1" ht="13.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A17" s="106" t="s">
         <v>65</v>
       </c>
@@ -7912,7 +7912,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="18" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="18" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A18" s="106" t="s">
         <v>65</v>
       </c>
@@ -7958,7 +7958,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="19" spans="1:20" s="5" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="19" spans="1:20" s="5" customFormat="1" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A19" s="106" t="s">
         <v>65</v>
       </c>
@@ -8004,7 +8004,7 @@
         <v>72</v>
       </c>
     </row>
-    <row r="20" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="20" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A20" s="106" t="s">
         <v>65</v>
       </c>
@@ -8062,7 +8062,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="21" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="21" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A21" s="106" t="s">
         <v>65</v>
       </c>
@@ -8120,7 +8120,7 @@
         <v>75</v>
       </c>
     </row>
-    <row r="22" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:20" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A22" s="106" t="s">
         <v>65</v>
       </c>
@@ -8174,7 +8174,7 @@
         <v>78</v>
       </c>
     </row>
-    <row r="23" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A23" s="113" t="s">
         <v>79</v>
       </c>
@@ -8232,7 +8232,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="24" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A24" s="106" t="s">
         <v>79</v>
       </c>
@@ -8290,7 +8290,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="25" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A25" s="106" t="s">
         <v>79</v>
       </c>
@@ -8406,7 +8406,7 @@
         <v>81</v>
       </c>
     </row>
-    <row r="27" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="27" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A27" s="106" t="s">
         <v>79</v>
       </c>
@@ -8446,7 +8446,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="28" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="28" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A28" s="106" t="s">
         <v>79</v>
       </c>
@@ -8488,7 +8488,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="29" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="29" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A29" s="106" t="s">
         <v>79</v>
       </c>
@@ -8530,7 +8530,7 @@
         <v>87</v>
       </c>
     </row>
-    <row r="30" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="30" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A30" s="106" t="s">
         <v>79</v>
       </c>
@@ -8572,7 +8572,7 @@
         <v>92</v>
       </c>
     </row>
-    <row r="31" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="31" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A31" s="106" t="s">
         <v>79</v>
       </c>
@@ -8614,7 +8614,7 @@
         <v>94</v>
       </c>
     </row>
-    <row r="32" spans="1:20" s="4" customFormat="1" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="32" spans="1:20" s="4" customFormat="1" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A32" s="106" t="s">
         <v>95</v>
       </c>
@@ -8656,7 +8656,7 @@
         <v>97</v>
       </c>
     </row>
-    <row r="33" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A33" s="113" t="s">
         <v>95</v>
       </c>
@@ -8710,7 +8710,7 @@
         <v>100</v>
       </c>
     </row>
-    <row r="34" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="34" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A34" s="107" t="s">
         <v>95</v>
       </c>
@@ -8752,7 +8752,7 @@
       <c r="S34" s="107"/>
       <c r="T34" s="111"/>
     </row>
-    <row r="35" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="35" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A35" s="106" t="s">
         <v>95</v>
       </c>
@@ -8856,7 +8856,7 @@
         <v>107</v>
       </c>
     </row>
-    <row r="37" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A37" s="132" t="s">
         <v>95</v>
       </c>
@@ -8910,7 +8910,7 @@
         <v>118</v>
       </c>
     </row>
-    <row r="38" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A38" s="113" t="s">
         <v>108</v>
       </c>
@@ -8992,7 +8992,7 @@
         <v>114</v>
       </c>
     </row>
-    <row r="40" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A40" s="106" t="s">
         <v>119</v>
       </c>
@@ -9036,7 +9036,7 @@
         <v>122</v>
       </c>
     </row>
-    <row r="41" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="41" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A41" s="106" t="s">
         <v>123</v>
       </c>
@@ -9094,7 +9094,7 @@
         <v>126</v>
       </c>
     </row>
-    <row r="42" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="42" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A42" s="106" t="s">
         <v>123</v>
       </c>
@@ -9152,7 +9152,7 @@
         <v>129</v>
       </c>
     </row>
-    <row r="43" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="43" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A43" s="106" t="s">
         <v>123</v>
       </c>
@@ -9198,7 +9198,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="44" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="44" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A44" s="106" t="s">
         <v>123</v>
       </c>
@@ -9244,7 +9244,7 @@
         <v>131</v>
       </c>
     </row>
-    <row r="45" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A45" s="113" t="s">
         <v>123</v>
       </c>
@@ -9295,7 +9295,7 @@
         <v>135</v>
       </c>
     </row>
-    <row r="46" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="46" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A46" s="106" t="s">
         <v>123</v>
       </c>
@@ -9355,7 +9355,7 @@
         <v>140</v>
       </c>
     </row>
-    <row r="47" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:20" ht="14.5" x14ac:dyDescent="0.35">
       <c r="A47" s="113" t="s">
         <v>141</v>
       </c>
@@ -9401,7 +9401,7 @@
         <v>145</v>
       </c>
     </row>
-    <row r="48" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="48" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A48" s="106" t="s">
         <v>146</v>
       </c>
@@ -9459,7 +9459,7 @@
         <v>149</v>
       </c>
     </row>
-    <row r="49" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A49" s="113" t="s">
         <v>150</v>
       </c>
@@ -9507,7 +9507,7 @@
         <v>153</v>
       </c>
     </row>
-    <row r="50" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A50" s="113" t="s">
         <v>154</v>
       </c>
@@ -9547,7 +9547,7 @@
         <v>157</v>
       </c>
     </row>
-    <row r="51" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A51" s="113" t="s">
         <v>154</v>
       </c>
@@ -9589,7 +9589,7 @@
         <v>160</v>
       </c>
     </row>
-    <row r="52" spans="1:20" s="4" customFormat="1" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="52" spans="1:20" s="4" customFormat="1" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A52" s="106" t="s">
         <v>161</v>
       </c>
@@ -9649,7 +9649,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="53" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="53" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A53" s="106" t="s">
         <v>161</v>
       </c>
@@ -9693,7 +9693,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="54" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="54" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A54" s="106" t="s">
         <v>161</v>
       </c>
@@ -9743,7 +9743,7 @@
         <v>166</v>
       </c>
     </row>
-    <row r="55" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="55" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A55" s="106" t="s">
         <v>161</v>
       </c>
@@ -9785,7 +9785,7 @@
         <v>168</v>
       </c>
     </row>
-    <row r="56" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A56" s="106" t="s">
         <v>169</v>
       </c>
@@ -9839,7 +9839,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="57" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="57" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A57" s="106" t="s">
         <v>169</v>
       </c>
@@ -9897,7 +9897,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="58" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="58" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A58" s="106" t="s">
         <v>169</v>
       </c>
@@ -9948,7 +9948,7 @@
         <v>171</v>
       </c>
     </row>
-    <row r="59" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="59" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A59" s="106" t="s">
         <v>174</v>
       </c>
@@ -10006,7 +10006,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="60" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="60" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A60" s="106" t="s">
         <v>178</v>
       </c>
@@ -10050,7 +10050,7 @@
         <v>181</v>
       </c>
     </row>
-    <row r="61" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="61" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A61" s="106" t="s">
         <v>182</v>
       </c>
@@ -10108,7 +10108,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="62" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="62" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A62" s="106" t="s">
         <v>182</v>
       </c>
@@ -10166,7 +10166,7 @@
         <v>188</v>
       </c>
     </row>
-    <row r="63" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="63" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A63" s="106" t="s">
         <v>182</v>
       </c>
@@ -10224,7 +10224,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="64" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A64" s="106" t="s">
         <v>182</v>
       </c>
@@ -10282,7 +10282,7 @@
         <v>191</v>
       </c>
     </row>
-    <row r="65" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="65" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A65" s="106" t="s">
         <v>182</v>
       </c>
@@ -10340,7 +10340,7 @@
         <v>185</v>
       </c>
     </row>
-    <row r="66" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="66" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A66" s="106" t="s">
         <v>182</v>
       </c>
@@ -10398,7 +10398,7 @@
         <v>195</v>
       </c>
     </row>
-    <row r="67" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="67" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A67" s="106" t="s">
         <v>182</v>
       </c>
@@ -10456,7 +10456,7 @@
         <v>199</v>
       </c>
     </row>
-    <row r="68" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="68" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A68" s="106" t="s">
         <v>200</v>
       </c>
@@ -10506,7 +10506,7 @@
         <v>203</v>
       </c>
     </row>
-    <row r="69" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="69" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A69" s="106" t="s">
         <v>200</v>
       </c>
@@ -10556,7 +10556,7 @@
         <v>206</v>
       </c>
     </row>
-    <row r="70" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="70" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A70" s="106" t="s">
         <v>200</v>
       </c>
@@ -10600,7 +10600,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="71" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="71" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A71" s="106" t="s">
         <v>200</v>
       </c>
@@ -10644,7 +10644,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="72" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="72" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A72" s="106" t="s">
         <v>200</v>
       </c>
@@ -10694,7 +10694,7 @@
         <v>209</v>
       </c>
     </row>
-    <row r="73" spans="1:20" ht="15" hidden="1" customHeight="1" x14ac:dyDescent="0.25">
+    <row r="73" spans="1:20" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="A73" s="106" t="s">
         <v>212</v>
       </c>
@@ -10752,7 +10752,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="74" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="74" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A74" s="106" t="s">
         <v>212</v>
       </c>
@@ -10801,7 +10801,7 @@
         <v>215</v>
       </c>
     </row>
-    <row r="75" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="75" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A75" s="106" t="s">
         <v>212</v>
       </c>
@@ -10859,7 +10859,7 @@
         <v>218</v>
       </c>
     </row>
-    <row r="76" spans="1:20" ht="14.5" hidden="1" x14ac:dyDescent="0.25">
+    <row r="76" spans="1:20" ht="14.5" x14ac:dyDescent="0.25">
       <c r="A76" s="106" t="s">
         <v>212</v>
       </c>
@@ -10917,7 +10917,7 @@
         <v>221</v>
       </c>
     </row>
-    <row r="77" spans="1:20" ht="15" hidden="1" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
+    <row r="77" spans="1:20" ht="15" customHeight="1" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A77" s="148" t="s">
         <v>212</v>
       </c>
@@ -10966,18 +10966,7 @@
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A3:T77" xr:uid="{00000000-0001-0000-0000-000000000000}">
-    <filterColumn colId="3">
-      <filters>
-        <filter val="planned"/>
-      </filters>
-    </filterColumn>
-    <filterColumn colId="5">
-      <filters>
-        <filter val="2024"/>
-      </filters>
-    </filterColumn>
-  </autoFilter>
+  <autoFilter ref="A3:T77" xr:uid="{00000000-0001-0000-0000-000000000000}"/>
   <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:T77">
     <sortCondition ref="A4:A77"/>
   </sortState>
@@ -13904,12 +13893,16 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="c2313526-4958-4054-bf54-a58bf530b099" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="715071c2-35c6-41f1-a6a3-03dd21313204">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -14165,22 +14158,22 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="c2313526-4958-4054-bf54-a58bf530b099" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="715071c2-35c6-41f1-a6a3-03dd21313204">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-    <_ip_UnifiedCompliancePolicyUIAction xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-    <_ip_UnifiedCompliancePolicyProperties xmlns="http://schemas.microsoft.com/sharepoint/v3" xsi:nil="true"/>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD84AF24-CD79-4A30-B9DC-32ADB805B515}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{747AE611-1440-4520-B03B-280DC23564C0}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="c2313526-4958-4054-bf54-a58bf530b099"/>
+    <ds:schemaRef ds:uri="715071c2-35c6-41f1-a6a3-03dd21313204"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -14206,13 +14199,9 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{747AE611-1440-4520-B03B-280DC23564C0}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BD84AF24-CD79-4A30-B9DC-32ADB805B515}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="c2313526-4958-4054-bf54-a58bf530b099"/>
-    <ds:schemaRef ds:uri="715071c2-35c6-41f1-a6a3-03dd21313204"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>